<commit_message>
Sync données pipeline depuis main (parquet, cross-check, legacy xlsx)
Rattrapage manuel des mises à jour automatiques publiées sur main
(seule branche où le pipeline tourne) : database_paris.parquet,
cross_check_log.csv, et les xlsx legacy Forecast-01072026-18Z (run
recomplété) / Forecast-02072026-12Z (nouveau run). Sauvegardes datées
du parquet et du xlsx écrasé conservées avant remplacement.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/legacy/Forecast-01072026-18Z.xlsx
+++ b/legacy/Forecast-01072026-18Z.xlsx
@@ -638,7 +638,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 02/07/2026 08:14</t>
+          <t>Généré le : 02/07/2026 22:56</t>
         </is>
       </c>
     </row>
@@ -1415,7 +1415,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X21"/>
+  <dimension ref="A1:W21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -1441,7 +1441,6 @@
     <col width="11" customWidth="1" min="21" max="21"/>
     <col width="11" customWidth="1" min="22" max="22"/>
     <col width="11" customWidth="1" min="23" max="23"/>
-    <col width="11" customWidth="1" min="24" max="24"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1454,7 +1453,7 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Généré le : 02/07/2026 08:14</t>
+          <t>Généré le : 02/07/2026 22:56</t>
         </is>
       </c>
     </row>
@@ -1579,11 +1578,6 @@
       <c r="W5" s="2" t="inlineStr">
         <is>
           <t>Δ 27-Jun 12Z</t>
-        </is>
-      </c>
-      <c r="X5" s="2" t="inlineStr">
-        <is>
-          <t>Δ 27-Jun 0Z</t>
         </is>
       </c>
     </row>
@@ -1659,9 +1653,6 @@
       <c r="W6" s="10" t="n">
         <v>0.6</v>
       </c>
-      <c r="X6" s="10" t="n">
-        <v>1</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n">
@@ -1735,9 +1726,6 @@
       <c r="W7" s="8" t="n">
         <v>-1.3</v>
       </c>
-      <c r="X7" s="8" t="n">
-        <v>-1.5</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n">
@@ -1811,9 +1799,6 @@
       <c r="W8" s="8" t="n">
         <v>-0.5</v>
       </c>
-      <c r="X8" s="10" t="n">
-        <v>0.7</v>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n">
@@ -1887,9 +1872,6 @@
       <c r="W9" s="10" t="n">
         <v>1.3</v>
       </c>
-      <c r="X9" s="10" t="n">
-        <v>1.8</v>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n">
@@ -1963,9 +1945,6 @@
       <c r="W10" s="10" t="n">
         <v>1.5</v>
       </c>
-      <c r="X10" s="10" t="n">
-        <v>2.5</v>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n">
@@ -2039,9 +2018,6 @@
       <c r="W11" s="8" t="n">
         <v>-1.2</v>
       </c>
-      <c r="X11" s="10" t="n">
-        <v>0.4</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n">
@@ -2115,9 +2091,6 @@
       <c r="W12" s="8" t="n">
         <v>-1.5</v>
       </c>
-      <c r="X12" s="8" t="n">
-        <v>-0.8</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n">
@@ -2191,9 +2164,6 @@
       <c r="W13" s="10" t="n">
         <v>1.4</v>
       </c>
-      <c r="X13" s="10" t="n">
-        <v>1.2</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n">
@@ -2267,9 +2237,6 @@
       <c r="W14" s="10" t="n">
         <v>2</v>
       </c>
-      <c r="X14" s="10" t="n">
-        <v>2.8</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n">
@@ -2343,9 +2310,6 @@
       <c r="W15" s="10" t="n">
         <v>1.1</v>
       </c>
-      <c r="X15" s="10" t="n">
-        <v>2.5</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n">
@@ -2419,9 +2383,6 @@
       <c r="W16" s="10" t="n">
         <v>0.3</v>
       </c>
-      <c r="X16" s="10" t="n">
-        <v>2</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n">
@@ -2495,9 +2456,6 @@
       <c r="W17" s="8" t="n">
         <v>-1.5</v>
       </c>
-      <c r="X17" s="7" t="n">
-        <v/>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n">
@@ -2571,9 +2529,6 @@
       <c r="W18" s="7" t="n">
         <v/>
       </c>
-      <c r="X18" s="7" t="n">
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n">
@@ -2647,9 +2602,6 @@
       <c r="W19" s="7" t="n">
         <v/>
       </c>
-      <c r="X19" s="7" t="n">
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n">
@@ -2723,9 +2675,6 @@
       <c r="W20" s="7" t="n">
         <v/>
       </c>
-      <c r="X20" s="7" t="n">
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n">
@@ -2797,9 +2746,6 @@
         <v/>
       </c>
       <c r="W21" s="7" t="n">
-        <v/>
-      </c>
-      <c r="X21" s="7" t="n">
         <v/>
       </c>
     </row>

</xml_diff>